<commit_message>
Actualizacion de Datos PROM
</commit_message>
<xml_diff>
--- a/data/CORTEPRIMERSEMESTRE2026.xlsx
+++ b/data/CORTEPRIMERSEMESTRE2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\IT Teacher\Documents\BOLETINES\Corte de Calificaciones\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF598D81-321B-4069-8745-E0C2D0F88837}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B45D3BAA-B657-4A7F-8A72-AC47836B5A0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="11370" xr2:uid="{A1D48B81-9DDC-468E-92F8-F1A357059321}"/>
+    <workbookView xWindow="2280" yWindow="2280" windowWidth="14400" windowHeight="8170" xr2:uid="{A1D48B81-9DDC-468E-92F8-F1A357059321}"/>
   </bookViews>
   <sheets>
     <sheet name="DB" sheetId="1" r:id="rId1"/>
@@ -1547,15 +1547,6 @@
     <t>Valdes</t>
   </si>
   <si>
-    <t>Freshman</t>
-  </si>
-  <si>
-    <t>Junior</t>
-  </si>
-  <si>
-    <t>Senior</t>
-  </si>
-  <si>
     <t>8-1102-238</t>
   </si>
   <si>
@@ -2070,6 +2061,15 @@
   </si>
   <si>
     <t>8-1086-2384</t>
+  </si>
+  <si>
+    <t>PROM 2028</t>
+  </si>
+  <si>
+    <t>PROM 2027</t>
+  </si>
+  <si>
+    <t>PROM 2026</t>
   </si>
 </sst>
 </file>
@@ -5677,7 +5677,7 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
       <c r="B2" t="s">
         <v>11</v>
@@ -5689,7 +5689,7 @@
         <v>13</v>
       </c>
       <c r="E2" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F2" s="154">
         <v>3</v>
@@ -5712,7 +5712,7 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
       <c r="B3" t="s">
         <v>14</v>
@@ -5724,7 +5724,7 @@
         <v>13</v>
       </c>
       <c r="E3" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F3" s="154">
         <v>3</v>
@@ -5747,7 +5747,7 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
       <c r="B4" t="s">
         <v>16</v>
@@ -5759,7 +5759,7 @@
         <v>13</v>
       </c>
       <c r="E4" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F4" s="154">
         <v>3</v>
@@ -5782,7 +5782,7 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>508</v>
+        <v>505</v>
       </c>
       <c r="B5" t="s">
         <v>18</v>
@@ -5794,7 +5794,7 @@
         <v>13</v>
       </c>
       <c r="E5" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F5" s="154">
         <v>2</v>
@@ -5817,7 +5817,7 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>509</v>
+        <v>506</v>
       </c>
       <c r="B6" t="s">
         <v>20</v>
@@ -5829,7 +5829,7 @@
         <v>13</v>
       </c>
       <c r="E6" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F6" s="154">
         <v>2</v>
@@ -5852,7 +5852,7 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>510</v>
+        <v>507</v>
       </c>
       <c r="B7" t="s">
         <v>22</v>
@@ -5864,7 +5864,7 @@
         <v>13</v>
       </c>
       <c r="E7" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F7" s="154">
         <v>4</v>
@@ -5887,7 +5887,7 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>511</v>
+        <v>508</v>
       </c>
       <c r="B8" t="s">
         <v>24</v>
@@ -5899,7 +5899,7 @@
         <v>13</v>
       </c>
       <c r="E8" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F8" s="154">
         <v>4</v>
@@ -5922,7 +5922,7 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>512</v>
+        <v>509</v>
       </c>
       <c r="B9" t="s">
         <v>26</v>
@@ -5934,7 +5934,7 @@
         <v>13</v>
       </c>
       <c r="E9" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F9" s="154">
         <v>3</v>
@@ -5957,7 +5957,7 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>513</v>
+        <v>510</v>
       </c>
       <c r="B10" t="s">
         <v>28</v>
@@ -5969,7 +5969,7 @@
         <v>13</v>
       </c>
       <c r="E10" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F10" s="154">
         <v>5</v>
@@ -5992,7 +5992,7 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>514</v>
+        <v>511</v>
       </c>
       <c r="B11" t="s">
         <v>30</v>
@@ -6004,7 +6004,7 @@
         <v>13</v>
       </c>
       <c r="E11" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F11" s="154">
         <v>3</v>
@@ -6027,7 +6027,7 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
       <c r="B12" t="s">
         <v>32</v>
@@ -6039,7 +6039,7 @@
         <v>13</v>
       </c>
       <c r="E12" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F12" s="154">
         <v>3</v>
@@ -6062,7 +6062,7 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>516</v>
+        <v>513</v>
       </c>
       <c r="B13" t="s">
         <v>34</v>
@@ -6074,7 +6074,7 @@
         <v>13</v>
       </c>
       <c r="E13" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F13" s="154">
         <v>2</v>
@@ -6097,7 +6097,7 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="B14" t="s">
         <v>36</v>
@@ -6109,7 +6109,7 @@
         <v>13</v>
       </c>
       <c r="E14" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F14" s="154">
         <v>2</v>
@@ -6132,7 +6132,7 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
       <c r="B15" t="s">
         <v>38</v>
@@ -6144,7 +6144,7 @@
         <v>13</v>
       </c>
       <c r="E15" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F15" s="154">
         <v>2</v>
@@ -6167,7 +6167,7 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
       <c r="B16" t="s">
         <v>40</v>
@@ -6179,7 +6179,7 @@
         <v>13</v>
       </c>
       <c r="E16" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F16" s="154">
         <v>3</v>
@@ -6202,7 +6202,7 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="B17" t="s">
         <v>42</v>
@@ -6214,7 +6214,7 @@
         <v>13</v>
       </c>
       <c r="E17" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F17" s="154">
         <v>3</v>
@@ -6237,7 +6237,7 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="B18" t="s">
         <v>32</v>
@@ -6249,7 +6249,7 @@
         <v>13</v>
       </c>
       <c r="E18" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F18" s="154">
         <v>5</v>
@@ -6272,7 +6272,7 @@
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="B19" t="s">
         <v>45</v>
@@ -6284,7 +6284,7 @@
         <v>13</v>
       </c>
       <c r="E19" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F19" s="154">
         <v>2</v>
@@ -6307,7 +6307,7 @@
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
       <c r="B20" t="s">
         <v>47</v>
@@ -6319,7 +6319,7 @@
         <v>13</v>
       </c>
       <c r="E20" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F20" s="154">
         <v>4</v>
@@ -6342,7 +6342,7 @@
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
       <c r="B21" t="s">
         <v>49</v>
@@ -6354,7 +6354,7 @@
         <v>13</v>
       </c>
       <c r="E21" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F21" s="154">
         <v>5</v>
@@ -6377,7 +6377,7 @@
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>525</v>
+        <v>522</v>
       </c>
       <c r="B22" t="s">
         <v>38</v>
@@ -6389,7 +6389,7 @@
         <v>13</v>
       </c>
       <c r="E22" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F22" s="154">
         <v>4</v>
@@ -6412,7 +6412,7 @@
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>526</v>
+        <v>523</v>
       </c>
       <c r="B23" t="s">
         <v>52</v>
@@ -6424,7 +6424,7 @@
         <v>13</v>
       </c>
       <c r="E23" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F23" s="154">
         <v>5</v>
@@ -6459,7 +6459,7 @@
         <v>13</v>
       </c>
       <c r="E24" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F24" s="154">
         <v>3</v>
@@ -6482,7 +6482,7 @@
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>527</v>
+        <v>524</v>
       </c>
       <c r="B25" t="s">
         <v>56</v>
@@ -6494,7 +6494,7 @@
         <v>13</v>
       </c>
       <c r="E25" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F25" s="154">
         <v>4</v>
@@ -6517,7 +6517,7 @@
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>528</v>
+        <v>525</v>
       </c>
       <c r="B26" t="s">
         <v>58</v>
@@ -6529,7 +6529,7 @@
         <v>13</v>
       </c>
       <c r="E26" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F26" s="154">
         <v>3</v>
@@ -6552,7 +6552,7 @@
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>529</v>
+        <v>526</v>
       </c>
       <c r="B27" t="s">
         <v>60</v>
@@ -6564,7 +6564,7 @@
         <v>13</v>
       </c>
       <c r="E27" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F27" s="154">
         <v>4</v>
@@ -6587,7 +6587,7 @@
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>530</v>
+        <v>527</v>
       </c>
       <c r="B28" t="s">
         <v>62</v>
@@ -6599,7 +6599,7 @@
         <v>13</v>
       </c>
       <c r="E28" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F28" s="154">
         <v>2</v>
@@ -6622,7 +6622,7 @@
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>531</v>
+        <v>528</v>
       </c>
       <c r="B29" t="s">
         <v>63</v>
@@ -6634,7 +6634,7 @@
         <v>13</v>
       </c>
       <c r="E29" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F29" s="154">
         <v>4</v>
@@ -6657,7 +6657,7 @@
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>532</v>
+        <v>529</v>
       </c>
       <c r="B30" t="s">
         <v>65</v>
@@ -6669,7 +6669,7 @@
         <v>13</v>
       </c>
       <c r="E30" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F30" s="154">
         <v>2</v>
@@ -6692,7 +6692,7 @@
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>533</v>
+        <v>530</v>
       </c>
       <c r="B31" t="s">
         <v>67</v>
@@ -6704,7 +6704,7 @@
         <v>13</v>
       </c>
       <c r="E31" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F31" s="154">
         <v>5</v>
@@ -6727,7 +6727,7 @@
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>534</v>
+        <v>531</v>
       </c>
       <c r="B32" t="s">
         <v>69</v>
@@ -6739,7 +6739,7 @@
         <v>13</v>
       </c>
       <c r="E32" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F32" s="154">
         <v>5</v>
@@ -6762,7 +6762,7 @@
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>535</v>
+        <v>532</v>
       </c>
       <c r="B33" t="s">
         <v>32</v>
@@ -6774,7 +6774,7 @@
         <v>72</v>
       </c>
       <c r="E33" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F33" s="154">
         <v>2</v>
@@ -6797,7 +6797,7 @@
     </row>
     <row r="34" spans="1:11" s="153" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>536</v>
+        <v>533</v>
       </c>
       <c r="B34" s="153" t="s">
         <v>73</v>
@@ -6808,8 +6808,8 @@
       <c r="D34" s="153" t="s">
         <v>72</v>
       </c>
-      <c r="E34" s="153" t="s">
-        <v>502</v>
+      <c r="E34" t="s">
+        <v>674</v>
       </c>
       <c r="F34" s="155">
         <v>4</v>
@@ -6832,7 +6832,7 @@
     </row>
     <row r="35" spans="1:11" s="153" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>537</v>
+        <v>534</v>
       </c>
       <c r="B35" s="153" t="s">
         <v>75</v>
@@ -6843,8 +6843,8 @@
       <c r="D35" s="153" t="s">
         <v>72</v>
       </c>
-      <c r="E35" s="153" t="s">
-        <v>502</v>
+      <c r="E35" t="s">
+        <v>674</v>
       </c>
       <c r="F35" s="155">
         <v>3</v>
@@ -6867,7 +6867,7 @@
     </row>
     <row r="36" spans="1:11" s="153" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>538</v>
+        <v>535</v>
       </c>
       <c r="B36" s="153" t="s">
         <v>76</v>
@@ -6878,8 +6878,8 @@
       <c r="D36" s="153" t="s">
         <v>72</v>
       </c>
-      <c r="E36" s="153" t="s">
-        <v>502</v>
+      <c r="E36" t="s">
+        <v>674</v>
       </c>
       <c r="F36" s="155">
         <v>2</v>
@@ -6902,7 +6902,7 @@
     </row>
     <row r="37" spans="1:11" s="153" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="B37" s="153" t="s">
         <v>78</v>
@@ -6913,8 +6913,8 @@
       <c r="D37" s="153" t="s">
         <v>72</v>
       </c>
-      <c r="E37" s="153" t="s">
-        <v>502</v>
+      <c r="E37" t="s">
+        <v>674</v>
       </c>
       <c r="F37" s="155">
         <v>3</v>
@@ -6937,7 +6937,7 @@
     </row>
     <row r="38" spans="1:11" s="153" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
       <c r="B38" s="153" t="s">
         <v>80</v>
@@ -6948,8 +6948,8 @@
       <c r="D38" s="153" t="s">
         <v>72</v>
       </c>
-      <c r="E38" s="153" t="s">
-        <v>502</v>
+      <c r="E38" t="s">
+        <v>674</v>
       </c>
       <c r="F38" s="155">
         <v>2</v>
@@ -6972,7 +6972,7 @@
     </row>
     <row r="39" spans="1:11" s="153" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="B39" s="153" t="s">
         <v>82</v>
@@ -6983,8 +6983,8 @@
       <c r="D39" s="153" t="s">
         <v>72</v>
       </c>
-      <c r="E39" s="153" t="s">
-        <v>502</v>
+      <c r="E39" t="s">
+        <v>674</v>
       </c>
       <c r="F39" s="155">
         <v>5</v>
@@ -7007,7 +7007,7 @@
     </row>
     <row r="40" spans="1:11" s="153" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
       <c r="B40" s="153" t="s">
         <v>83</v>
@@ -7018,8 +7018,8 @@
       <c r="D40" s="153" t="s">
         <v>72</v>
       </c>
-      <c r="E40" s="153" t="s">
-        <v>502</v>
+      <c r="E40" t="s">
+        <v>674</v>
       </c>
       <c r="F40" s="155">
         <v>4</v>
@@ -7042,7 +7042,7 @@
     </row>
     <row r="41" spans="1:11" s="153" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>543</v>
+        <v>540</v>
       </c>
       <c r="B41" s="153" t="s">
         <v>85</v>
@@ -7053,8 +7053,8 @@
       <c r="D41" s="153" t="s">
         <v>72</v>
       </c>
-      <c r="E41" s="153" t="s">
-        <v>502</v>
+      <c r="E41" t="s">
+        <v>674</v>
       </c>
       <c r="F41" s="155">
         <v>2</v>
@@ -7077,7 +7077,7 @@
     </row>
     <row r="42" spans="1:11" s="153" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>544</v>
+        <v>541</v>
       </c>
       <c r="B42" s="153" t="s">
         <v>87</v>
@@ -7088,8 +7088,8 @@
       <c r="D42" s="153" t="s">
         <v>72</v>
       </c>
-      <c r="E42" s="153" t="s">
-        <v>502</v>
+      <c r="E42" t="s">
+        <v>674</v>
       </c>
       <c r="F42" s="155">
         <v>5</v>
@@ -7112,7 +7112,7 @@
     </row>
     <row r="43" spans="1:11" s="153" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>545</v>
+        <v>542</v>
       </c>
       <c r="B43" s="153" t="s">
         <v>89</v>
@@ -7123,8 +7123,8 @@
       <c r="D43" s="153" t="s">
         <v>72</v>
       </c>
-      <c r="E43" s="153" t="s">
-        <v>502</v>
+      <c r="E43" t="s">
+        <v>674</v>
       </c>
       <c r="F43" s="155">
         <v>4</v>
@@ -7147,7 +7147,7 @@
     </row>
     <row r="44" spans="1:11" s="153" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>546</v>
+        <v>543</v>
       </c>
       <c r="B44" s="153" t="s">
         <v>91</v>
@@ -7158,8 +7158,8 @@
       <c r="D44" s="153" t="s">
         <v>72</v>
       </c>
-      <c r="E44" s="153" t="s">
-        <v>502</v>
+      <c r="E44" t="s">
+        <v>674</v>
       </c>
       <c r="F44" s="155">
         <v>3</v>
@@ -7182,7 +7182,7 @@
     </row>
     <row r="45" spans="1:11" s="153" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="B45" s="153" t="s">
         <v>83</v>
@@ -7193,8 +7193,8 @@
       <c r="D45" s="153" t="s">
         <v>72</v>
       </c>
-      <c r="E45" s="153" t="s">
-        <v>502</v>
+      <c r="E45" t="s">
+        <v>674</v>
       </c>
       <c r="F45" s="155">
         <v>4</v>
@@ -7217,7 +7217,7 @@
     </row>
     <row r="46" spans="1:11" s="153" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>548</v>
+        <v>545</v>
       </c>
       <c r="B46" s="153" t="s">
         <v>94</v>
@@ -7228,8 +7228,8 @@
       <c r="D46" s="153" t="s">
         <v>72</v>
       </c>
-      <c r="E46" s="153" t="s">
-        <v>502</v>
+      <c r="E46" t="s">
+        <v>674</v>
       </c>
       <c r="F46" s="155">
         <v>3</v>
@@ -7252,7 +7252,7 @@
     </row>
     <row r="47" spans="1:11" s="153" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="B47" s="153" t="s">
         <v>96</v>
@@ -7263,8 +7263,8 @@
       <c r="D47" s="153" t="s">
         <v>72</v>
       </c>
-      <c r="E47" s="153" t="s">
-        <v>502</v>
+      <c r="E47" t="s">
+        <v>674</v>
       </c>
       <c r="F47" s="155">
         <v>4</v>
@@ -7287,7 +7287,7 @@
     </row>
     <row r="48" spans="1:11" s="153" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>550</v>
+        <v>547</v>
       </c>
       <c r="B48" s="153" t="s">
         <v>98</v>
@@ -7298,8 +7298,8 @@
       <c r="D48" s="153" t="s">
         <v>72</v>
       </c>
-      <c r="E48" s="153" t="s">
-        <v>502</v>
+      <c r="E48" t="s">
+        <v>674</v>
       </c>
       <c r="F48" s="155">
         <v>5</v>
@@ -7322,7 +7322,7 @@
     </row>
     <row r="49" spans="1:11" s="153" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
       <c r="B49" s="153" t="s">
         <v>36</v>
@@ -7333,8 +7333,8 @@
       <c r="D49" s="153" t="s">
         <v>72</v>
       </c>
-      <c r="E49" s="153" t="s">
-        <v>502</v>
+      <c r="E49" t="s">
+        <v>674</v>
       </c>
       <c r="F49" s="155">
         <v>3</v>
@@ -7357,7 +7357,7 @@
     </row>
     <row r="50" spans="1:11" s="153" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>552</v>
+        <v>549</v>
       </c>
       <c r="B50" s="153" t="s">
         <v>101</v>
@@ -7368,8 +7368,8 @@
       <c r="D50" s="153" t="s">
         <v>72</v>
       </c>
-      <c r="E50" s="153" t="s">
-        <v>502</v>
+      <c r="E50" t="s">
+        <v>674</v>
       </c>
       <c r="F50" s="155">
         <v>3</v>
@@ -7389,7 +7389,7 @@
     </row>
     <row r="51" spans="1:11" s="153" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>553</v>
+        <v>550</v>
       </c>
       <c r="B51" s="153" t="s">
         <v>103</v>
@@ -7400,8 +7400,8 @@
       <c r="D51" s="153" t="s">
         <v>72</v>
       </c>
-      <c r="E51" s="153" t="s">
-        <v>502</v>
+      <c r="E51" t="s">
+        <v>674</v>
       </c>
       <c r="F51" s="155">
         <v>3</v>
@@ -7424,7 +7424,7 @@
     </row>
     <row r="52" spans="1:11" s="153" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>554</v>
+        <v>551</v>
       </c>
       <c r="B52" s="153" t="s">
         <v>54</v>
@@ -7435,8 +7435,8 @@
       <c r="D52" s="153" t="s">
         <v>72</v>
       </c>
-      <c r="E52" s="153" t="s">
-        <v>502</v>
+      <c r="E52" t="s">
+        <v>674</v>
       </c>
       <c r="F52" s="155">
         <v>3</v>
@@ -7459,7 +7459,7 @@
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>555</v>
+        <v>552</v>
       </c>
       <c r="B53" t="s">
         <v>105</v>
@@ -7471,7 +7471,7 @@
         <v>72</v>
       </c>
       <c r="E53" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F53" s="154">
         <v>2</v>
@@ -7494,7 +7494,7 @@
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>556</v>
+        <v>553</v>
       </c>
       <c r="B54" t="s">
         <v>107</v>
@@ -7506,7 +7506,7 @@
         <v>72</v>
       </c>
       <c r="E54" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F54" s="154">
         <v>2</v>
@@ -7529,7 +7529,7 @@
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>557</v>
+        <v>554</v>
       </c>
       <c r="B55" t="s">
         <v>109</v>
@@ -7541,7 +7541,7 @@
         <v>72</v>
       </c>
       <c r="E55" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F55" s="154">
         <v>4</v>
@@ -7564,7 +7564,7 @@
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>558</v>
+        <v>555</v>
       </c>
       <c r="B56" t="s">
         <v>111</v>
@@ -7576,7 +7576,7 @@
         <v>72</v>
       </c>
       <c r="E56" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F56" s="154">
         <v>2</v>
@@ -7599,7 +7599,7 @@
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>559</v>
+        <v>556</v>
       </c>
       <c r="B57" t="s">
         <v>113</v>
@@ -7611,7 +7611,7 @@
         <v>72</v>
       </c>
       <c r="E57" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F57" s="154">
         <v>3</v>
@@ -7634,7 +7634,7 @@
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>560</v>
+        <v>557</v>
       </c>
       <c r="B58" t="s">
         <v>115</v>
@@ -7646,7 +7646,7 @@
         <v>72</v>
       </c>
       <c r="E58" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F58" s="154">
         <v>5</v>
@@ -7669,7 +7669,7 @@
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>561</v>
+        <v>558</v>
       </c>
       <c r="B59" t="s">
         <v>38</v>
@@ -7681,7 +7681,7 @@
         <v>72</v>
       </c>
       <c r="E59" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F59" s="154">
         <v>2</v>
@@ -7704,7 +7704,7 @@
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>562</v>
+        <v>559</v>
       </c>
       <c r="B60" t="s">
         <v>118</v>
@@ -7716,7 +7716,7 @@
         <v>72</v>
       </c>
       <c r="E60" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F60" s="154">
         <v>4</v>
@@ -7739,7 +7739,7 @@
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="B61" t="s">
         <v>120</v>
@@ -7751,7 +7751,7 @@
         <v>72</v>
       </c>
       <c r="E61" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F61" s="154">
         <v>3</v>
@@ -7774,7 +7774,7 @@
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="B62" t="s">
         <v>122</v>
@@ -7786,7 +7786,7 @@
         <v>72</v>
       </c>
       <c r="E62" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F62" s="154">
         <v>4</v>
@@ -7809,7 +7809,7 @@
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>565</v>
+        <v>562</v>
       </c>
       <c r="B63" t="s">
         <v>124</v>
@@ -7821,7 +7821,7 @@
         <v>72</v>
       </c>
       <c r="E63" t="s">
-        <v>502</v>
+        <v>674</v>
       </c>
       <c r="F63" s="154">
         <v>2</v>
@@ -7844,7 +7844,7 @@
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>566</v>
+        <v>563</v>
       </c>
       <c r="B64" t="s">
         <v>126</v>
@@ -7856,7 +7856,7 @@
         <v>13</v>
       </c>
       <c r="E64" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F64" s="154">
         <v>3</v>
@@ -7879,7 +7879,7 @@
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>567</v>
+        <v>564</v>
       </c>
       <c r="B65" t="s">
         <v>98</v>
@@ -7891,7 +7891,7 @@
         <v>13</v>
       </c>
       <c r="E65" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F65" s="154">
         <v>2</v>
@@ -7914,7 +7914,7 @@
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>568</v>
+        <v>565</v>
       </c>
       <c r="B66" t="s">
         <v>129</v>
@@ -7926,7 +7926,7 @@
         <v>13</v>
       </c>
       <c r="E66" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F66" s="154">
         <v>2</v>
@@ -7949,7 +7949,7 @@
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>569</v>
+        <v>566</v>
       </c>
       <c r="B67" t="s">
         <v>131</v>
@@ -7961,7 +7961,7 @@
         <v>13</v>
       </c>
       <c r="E67" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F67" s="154">
         <v>4</v>
@@ -7984,7 +7984,7 @@
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
-        <v>570</v>
+        <v>567</v>
       </c>
       <c r="B68" t="s">
         <v>133</v>
@@ -7996,7 +7996,7 @@
         <v>13</v>
       </c>
       <c r="E68" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F68" s="154">
         <v>3</v>
@@ -8019,7 +8019,7 @@
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>571</v>
+        <v>568</v>
       </c>
       <c r="B69" t="s">
         <v>135</v>
@@ -8031,7 +8031,7 @@
         <v>13</v>
       </c>
       <c r="E69" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F69" s="154">
         <v>2</v>
@@ -8054,7 +8054,7 @@
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
       <c r="B70" t="s">
         <v>14</v>
@@ -8066,7 +8066,7 @@
         <v>13</v>
       </c>
       <c r="E70" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F70" s="154">
         <v>3</v>
@@ -8089,7 +8089,7 @@
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>573</v>
+        <v>570</v>
       </c>
       <c r="B71" t="s">
         <v>11</v>
@@ -8101,7 +8101,7 @@
         <v>13</v>
       </c>
       <c r="E71" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F71" s="154">
         <v>5</v>
@@ -8124,7 +8124,7 @@
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>574</v>
+        <v>571</v>
       </c>
       <c r="B72" t="s">
         <v>137</v>
@@ -8136,7 +8136,7 @@
         <v>13</v>
       </c>
       <c r="E72" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F72" s="154">
         <v>3</v>
@@ -8159,7 +8159,7 @@
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="B73" t="s">
         <v>138</v>
@@ -8171,7 +8171,7 @@
         <v>13</v>
       </c>
       <c r="E73" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F73" s="154">
         <v>5</v>
@@ -8194,7 +8194,7 @@
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>576</v>
+        <v>573</v>
       </c>
       <c r="B74" t="s">
         <v>139</v>
@@ -8206,7 +8206,7 @@
         <v>13</v>
       </c>
       <c r="E74" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F74" s="154">
         <v>4</v>
@@ -8229,7 +8229,7 @@
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>577</v>
+        <v>574</v>
       </c>
       <c r="B75" t="s">
         <v>141</v>
@@ -8241,7 +8241,7 @@
         <v>13</v>
       </c>
       <c r="E75" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F75" s="154">
         <v>4</v>
@@ -8264,7 +8264,7 @@
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>578</v>
+        <v>575</v>
       </c>
       <c r="B76" t="s">
         <v>142</v>
@@ -8276,7 +8276,7 @@
         <v>13</v>
       </c>
       <c r="E76" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F76" s="154">
         <v>4</v>
@@ -8299,7 +8299,7 @@
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>579</v>
+        <v>576</v>
       </c>
       <c r="B77" t="s">
         <v>144</v>
@@ -8311,7 +8311,7 @@
         <v>13</v>
       </c>
       <c r="E77" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F77" s="154">
         <v>2</v>
@@ -8334,7 +8334,7 @@
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
-        <v>580</v>
+        <v>577</v>
       </c>
       <c r="B78" t="s">
         <v>145</v>
@@ -8346,7 +8346,7 @@
         <v>13</v>
       </c>
       <c r="E78" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F78" s="154">
         <v>3</v>
@@ -8369,7 +8369,7 @@
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
-        <v>581</v>
+        <v>578</v>
       </c>
       <c r="B79" t="s">
         <v>147</v>
@@ -8381,7 +8381,7 @@
         <v>13</v>
       </c>
       <c r="E79" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F79" s="154">
         <v>4</v>
@@ -8404,7 +8404,7 @@
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
-        <v>582</v>
+        <v>579</v>
       </c>
       <c r="B80" t="s">
         <v>149</v>
@@ -8416,7 +8416,7 @@
         <v>13</v>
       </c>
       <c r="E80" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F80" s="154">
         <v>5</v>
@@ -8439,7 +8439,7 @@
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="B81" t="s">
         <v>151</v>
@@ -8451,7 +8451,7 @@
         <v>13</v>
       </c>
       <c r="E81" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F81" s="154">
         <v>2</v>
@@ -8474,7 +8474,7 @@
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
-        <v>584</v>
+        <v>581</v>
       </c>
       <c r="B82" t="s">
         <v>56</v>
@@ -8486,7 +8486,7 @@
         <v>13</v>
       </c>
       <c r="E82" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F82" s="154">
         <v>3</v>
@@ -8509,7 +8509,7 @@
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
-        <v>585</v>
+        <v>582</v>
       </c>
       <c r="B83" t="s">
         <v>135</v>
@@ -8521,7 +8521,7 @@
         <v>13</v>
       </c>
       <c r="E83" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F83" s="154">
         <v>4</v>
@@ -8544,7 +8544,7 @@
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
       <c r="B84" t="s">
         <v>153</v>
@@ -8556,7 +8556,7 @@
         <v>13</v>
       </c>
       <c r="E84" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F84" s="154">
         <v>2</v>
@@ -8579,7 +8579,7 @@
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
-        <v>587</v>
+        <v>584</v>
       </c>
       <c r="B85" t="s">
         <v>155</v>
@@ -8591,7 +8591,7 @@
         <v>13</v>
       </c>
       <c r="E85" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F85" s="154">
         <v>5</v>
@@ -8614,7 +8614,7 @@
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
-        <v>588</v>
+        <v>585</v>
       </c>
       <c r="B86" t="s">
         <v>156</v>
@@ -8626,7 +8626,7 @@
         <v>13</v>
       </c>
       <c r="E86" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F86" s="154">
         <v>4</v>
@@ -8649,7 +8649,7 @@
     </row>
     <row r="87" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
-        <v>589</v>
+        <v>586</v>
       </c>
       <c r="B87" t="s">
         <v>158</v>
@@ -8661,7 +8661,7 @@
         <v>13</v>
       </c>
       <c r="E87" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F87" s="154">
         <v>5</v>
@@ -8684,7 +8684,7 @@
     </row>
     <row r="88" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
-        <v>590</v>
+        <v>587</v>
       </c>
       <c r="B88" t="s">
         <v>160</v>
@@ -8696,7 +8696,7 @@
         <v>13</v>
       </c>
       <c r="E88" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F88" s="154">
         <v>5</v>
@@ -8719,7 +8719,7 @@
     </row>
     <row r="89" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
-        <v>591</v>
+        <v>588</v>
       </c>
       <c r="B89" t="s">
         <v>162</v>
@@ -8731,7 +8731,7 @@
         <v>13</v>
       </c>
       <c r="E89" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F89" s="154">
         <v>3</v>
@@ -8754,7 +8754,7 @@
     </row>
     <row r="90" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
-        <v>592</v>
+        <v>589</v>
       </c>
       <c r="B90" t="s">
         <v>164</v>
@@ -8766,7 +8766,7 @@
         <v>13</v>
       </c>
       <c r="E90" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F90" s="154">
         <v>3</v>
@@ -8801,7 +8801,7 @@
         <v>13</v>
       </c>
       <c r="E91" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F91" s="154">
         <v>3</v>
@@ -8824,7 +8824,7 @@
     </row>
     <row r="92" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
-        <v>593</v>
+        <v>590</v>
       </c>
       <c r="B92" t="s">
         <v>54</v>
@@ -8836,7 +8836,7 @@
         <v>13</v>
       </c>
       <c r="E92" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F92" s="154">
         <v>4</v>
@@ -8859,7 +8859,7 @@
     </row>
     <row r="93" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
-        <v>594</v>
+        <v>591</v>
       </c>
       <c r="B93" t="s">
         <v>169</v>
@@ -8871,7 +8871,7 @@
         <v>72</v>
       </c>
       <c r="E93" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F93" s="154">
         <v>3</v>
@@ -8894,7 +8894,7 @@
     </row>
     <row r="94" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
-        <v>595</v>
+        <v>592</v>
       </c>
       <c r="B94" t="s">
         <v>171</v>
@@ -8906,7 +8906,7 @@
         <v>72</v>
       </c>
       <c r="E94" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F94" s="154">
         <v>5</v>
@@ -8929,7 +8929,7 @@
     </row>
     <row r="95" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
-        <v>596</v>
+        <v>593</v>
       </c>
       <c r="B95" t="s">
         <v>173</v>
@@ -8941,7 +8941,7 @@
         <v>72</v>
       </c>
       <c r="E95" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F95" s="154">
         <v>3</v>
@@ -8964,7 +8964,7 @@
     </row>
     <row r="96" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
-        <v>597</v>
+        <v>594</v>
       </c>
       <c r="B96" t="s">
         <v>175</v>
@@ -8976,7 +8976,7 @@
         <v>72</v>
       </c>
       <c r="E96" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F96" s="154">
         <v>3</v>
@@ -8999,7 +8999,7 @@
     </row>
     <row r="97" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
-        <v>598</v>
+        <v>595</v>
       </c>
       <c r="B97" t="s">
         <v>177</v>
@@ -9011,7 +9011,7 @@
         <v>72</v>
       </c>
       <c r="E97" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F97" s="154">
         <v>4</v>
@@ -9034,7 +9034,7 @@
     </row>
     <row r="98" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
-        <v>599</v>
+        <v>596</v>
       </c>
       <c r="B98" t="s">
         <v>179</v>
@@ -9046,7 +9046,7 @@
         <v>72</v>
       </c>
       <c r="E98" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F98" s="154">
         <v>2</v>
@@ -9069,7 +9069,7 @@
     </row>
     <row r="99" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
-        <v>600</v>
+        <v>597</v>
       </c>
       <c r="B99" t="s">
         <v>181</v>
@@ -9081,7 +9081,7 @@
         <v>72</v>
       </c>
       <c r="E99" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F99" s="154">
         <v>4</v>
@@ -9104,7 +9104,7 @@
     </row>
     <row r="100" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
-        <v>601</v>
+        <v>598</v>
       </c>
       <c r="B100" t="s">
         <v>182</v>
@@ -9116,7 +9116,7 @@
         <v>72</v>
       </c>
       <c r="E100" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F100" s="154">
         <v>4</v>
@@ -9139,7 +9139,7 @@
     </row>
     <row r="101" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
-        <v>602</v>
+        <v>599</v>
       </c>
       <c r="B101" t="s">
         <v>184</v>
@@ -9151,7 +9151,7 @@
         <v>72</v>
       </c>
       <c r="E101" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F101" s="154">
         <v>5</v>
@@ -9174,7 +9174,7 @@
     </row>
     <row r="102" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
-        <v>603</v>
+        <v>600</v>
       </c>
       <c r="B102" t="s">
         <v>185</v>
@@ -9186,7 +9186,7 @@
         <v>72</v>
       </c>
       <c r="E102" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F102" s="154">
         <v>5</v>
@@ -9209,7 +9209,7 @@
     </row>
     <row r="103" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
-        <v>604</v>
+        <v>601</v>
       </c>
       <c r="B103" t="s">
         <v>186</v>
@@ -9221,7 +9221,7 @@
         <v>72</v>
       </c>
       <c r="E103" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F103" s="154">
         <v>5</v>
@@ -9244,7 +9244,7 @@
     </row>
     <row r="104" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
-        <v>605</v>
+        <v>602</v>
       </c>
       <c r="B104" t="s">
         <v>188</v>
@@ -9256,7 +9256,7 @@
         <v>72</v>
       </c>
       <c r="E104" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F104" s="154">
         <v>4</v>
@@ -9279,7 +9279,7 @@
     </row>
     <row r="105" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
-        <v>606</v>
+        <v>603</v>
       </c>
       <c r="B105" t="s">
         <v>190</v>
@@ -9291,7 +9291,7 @@
         <v>72</v>
       </c>
       <c r="E105" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F105" s="154">
         <v>4</v>
@@ -9314,7 +9314,7 @@
     </row>
     <row r="106" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
-        <v>607</v>
+        <v>604</v>
       </c>
       <c r="B106" t="s">
         <v>192</v>
@@ -9326,7 +9326,7 @@
         <v>72</v>
       </c>
       <c r="E106" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F106" s="154">
         <v>5</v>
@@ -9361,7 +9361,7 @@
         <v>72</v>
       </c>
       <c r="E107" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F107" s="154">
         <v>3</v>
@@ -9384,7 +9384,7 @@
     </row>
     <row r="108" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
-        <v>608</v>
+        <v>605</v>
       </c>
       <c r="B108" t="s">
         <v>196</v>
@@ -9396,7 +9396,7 @@
         <v>72</v>
       </c>
       <c r="E108" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F108" s="154">
         <v>3</v>
@@ -9419,7 +9419,7 @@
     </row>
     <row r="109" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
-        <v>609</v>
+        <v>606</v>
       </c>
       <c r="B109" t="s">
         <v>197</v>
@@ -9431,7 +9431,7 @@
         <v>72</v>
       </c>
       <c r="E109" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F109" s="154">
         <v>2</v>
@@ -9454,7 +9454,7 @@
     </row>
     <row r="110" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
-        <v>610</v>
+        <v>607</v>
       </c>
       <c r="B110" t="s">
         <v>199</v>
@@ -9466,7 +9466,7 @@
         <v>72</v>
       </c>
       <c r="E110" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F110" s="154">
         <v>5</v>
@@ -9489,7 +9489,7 @@
     </row>
     <row r="111" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
-        <v>611</v>
+        <v>608</v>
       </c>
       <c r="B111" t="s">
         <v>200</v>
@@ -9501,7 +9501,7 @@
         <v>72</v>
       </c>
       <c r="E111" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F111" s="154">
         <v>3</v>
@@ -9524,7 +9524,7 @@
     </row>
     <row r="112" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
-        <v>612</v>
+        <v>609</v>
       </c>
       <c r="B112" t="s">
         <v>202</v>
@@ -9536,7 +9536,7 @@
         <v>72</v>
       </c>
       <c r="E112" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F112" s="154">
         <v>3</v>
@@ -9559,7 +9559,7 @@
     </row>
     <row r="113" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
-        <v>613</v>
+        <v>610</v>
       </c>
       <c r="B113" t="s">
         <v>204</v>
@@ -9571,7 +9571,7 @@
         <v>72</v>
       </c>
       <c r="E113" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F113" s="154">
         <v>4</v>
@@ -9594,7 +9594,7 @@
     </row>
     <row r="114" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
-        <v>614</v>
+        <v>611</v>
       </c>
       <c r="B114" t="s">
         <v>14</v>
@@ -9606,7 +9606,7 @@
         <v>72</v>
       </c>
       <c r="E114" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F114" s="154">
         <v>4</v>
@@ -9629,7 +9629,7 @@
     </row>
     <row r="115" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="B115" t="s">
         <v>205</v>
@@ -9641,7 +9641,7 @@
         <v>72</v>
       </c>
       <c r="E115" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F115" s="154">
         <v>2</v>
@@ -9664,7 +9664,7 @@
     </row>
     <row r="116" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
-        <v>616</v>
+        <v>613</v>
       </c>
       <c r="B116" t="s">
         <v>206</v>
@@ -9676,7 +9676,7 @@
         <v>72</v>
       </c>
       <c r="E116" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F116" s="154">
         <v>5</v>
@@ -9699,7 +9699,7 @@
     </row>
     <row r="117" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="B117" t="s">
         <v>207</v>
@@ -9711,7 +9711,7 @@
         <v>72</v>
       </c>
       <c r="E117" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F117" s="154">
         <v>4</v>
@@ -9734,7 +9734,7 @@
     </row>
     <row r="118" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
-        <v>618</v>
+        <v>615</v>
       </c>
       <c r="B118" t="s">
         <v>208</v>
@@ -9746,7 +9746,7 @@
         <v>72</v>
       </c>
       <c r="E118" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F118" s="154">
         <v>2</v>
@@ -9769,7 +9769,7 @@
     </row>
     <row r="119" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
-        <v>619</v>
+        <v>616</v>
       </c>
       <c r="B119" t="s">
         <v>210</v>
@@ -9781,7 +9781,7 @@
         <v>72</v>
       </c>
       <c r="E119" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F119" s="154">
         <v>2</v>
@@ -9804,7 +9804,7 @@
     </row>
     <row r="120" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
-        <v>620</v>
+        <v>617</v>
       </c>
       <c r="B120" t="s">
         <v>211</v>
@@ -9816,7 +9816,7 @@
         <v>72</v>
       </c>
       <c r="E120" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F120" s="154">
         <v>4</v>
@@ -9839,7 +9839,7 @@
     </row>
     <row r="121" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
-        <v>621</v>
+        <v>618</v>
       </c>
       <c r="B121" t="s">
         <v>212</v>
@@ -9851,7 +9851,7 @@
         <v>72</v>
       </c>
       <c r="E121" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F121" s="154">
         <v>3</v>
@@ -9874,7 +9874,7 @@
     </row>
     <row r="122" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
-        <v>622</v>
+        <v>619</v>
       </c>
       <c r="B122" t="s">
         <v>214</v>
@@ -9886,7 +9886,7 @@
         <v>72</v>
       </c>
       <c r="E122" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F122" s="154">
         <v>2</v>
@@ -9909,7 +9909,7 @@
     </row>
     <row r="123" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
-        <v>623</v>
+        <v>620</v>
       </c>
       <c r="B123" t="s">
         <v>216</v>
@@ -9921,7 +9921,7 @@
         <v>72</v>
       </c>
       <c r="E123" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="F123" s="154">
         <v>4</v>
@@ -9944,7 +9944,7 @@
     </row>
     <row r="124" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
-        <v>624</v>
+        <v>621</v>
       </c>
       <c r="B124" t="s">
         <v>217</v>
@@ -9956,7 +9956,7 @@
         <v>13</v>
       </c>
       <c r="E124" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F124" s="154">
         <v>5</v>
@@ -9979,7 +9979,7 @@
     </row>
     <row r="125" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
-        <v>625</v>
+        <v>622</v>
       </c>
       <c r="B125" t="s">
         <v>218</v>
@@ -9991,7 +9991,7 @@
         <v>13</v>
       </c>
       <c r="E125" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F125" s="154">
         <v>3</v>
@@ -10014,7 +10014,7 @@
     </row>
     <row r="126" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
-        <v>626</v>
+        <v>623</v>
       </c>
       <c r="B126" t="s">
         <v>220</v>
@@ -10026,7 +10026,7 @@
         <v>13</v>
       </c>
       <c r="E126" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F126" s="154">
         <v>2</v>
@@ -10049,7 +10049,7 @@
     </row>
     <row r="127" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
-        <v>627</v>
+        <v>624</v>
       </c>
       <c r="B127" t="s">
         <v>222</v>
@@ -10061,7 +10061,7 @@
         <v>13</v>
       </c>
       <c r="E127" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F127" s="154">
         <v>5</v>
@@ -10084,7 +10084,7 @@
     </row>
     <row r="128" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
-        <v>628</v>
+        <v>625</v>
       </c>
       <c r="B128" t="s">
         <v>185</v>
@@ -10096,7 +10096,7 @@
         <v>13</v>
       </c>
       <c r="E128" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F128" s="154">
         <v>5</v>
@@ -10119,7 +10119,7 @@
     </row>
     <row r="129" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
-        <v>629</v>
+        <v>626</v>
       </c>
       <c r="B129" t="s">
         <v>16</v>
@@ -10131,7 +10131,7 @@
         <v>13</v>
       </c>
       <c r="E129" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F129" s="154">
         <v>2</v>
@@ -10154,7 +10154,7 @@
     </row>
     <row r="130" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
-        <v>630</v>
+        <v>627</v>
       </c>
       <c r="B130" t="s">
         <v>20</v>
@@ -10166,7 +10166,7 @@
         <v>13</v>
       </c>
       <c r="E130" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F130" s="154">
         <v>3</v>
@@ -10189,7 +10189,7 @@
     </row>
     <row r="131" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
-        <v>631</v>
+        <v>628</v>
       </c>
       <c r="B131" t="s">
         <v>226</v>
@@ -10201,7 +10201,7 @@
         <v>13</v>
       </c>
       <c r="E131" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F131" s="154">
         <v>2</v>
@@ -10224,7 +10224,7 @@
     </row>
     <row r="132" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="B132" t="s">
         <v>228</v>
@@ -10236,7 +10236,7 @@
         <v>13</v>
       </c>
       <c r="E132" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F132" s="154">
         <v>4</v>
@@ -10259,7 +10259,7 @@
     </row>
     <row r="133" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="B133" t="s">
         <v>230</v>
@@ -10271,7 +10271,7 @@
         <v>13</v>
       </c>
       <c r="E133" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F133" s="154">
         <v>5</v>
@@ -10294,7 +10294,7 @@
     </row>
     <row r="134" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
-        <v>634</v>
+        <v>631</v>
       </c>
       <c r="B134" t="s">
         <v>151</v>
@@ -10306,7 +10306,7 @@
         <v>13</v>
       </c>
       <c r="E134" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F134" s="154">
         <v>2</v>
@@ -10329,7 +10329,7 @@
     </row>
     <row r="135" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
-        <v>635</v>
+        <v>632</v>
       </c>
       <c r="B135" t="s">
         <v>233</v>
@@ -10341,7 +10341,7 @@
         <v>13</v>
       </c>
       <c r="E135" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F135" s="154">
         <v>4</v>
@@ -10364,7 +10364,7 @@
     </row>
     <row r="136" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
-        <v>636</v>
+        <v>633</v>
       </c>
       <c r="B136" t="s">
         <v>234</v>
@@ -10376,7 +10376,7 @@
         <v>13</v>
       </c>
       <c r="E136" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F136" s="154">
         <v>4</v>
@@ -10399,7 +10399,7 @@
     </row>
     <row r="137" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
-        <v>637</v>
+        <v>634</v>
       </c>
       <c r="B137" t="s">
         <v>185</v>
@@ -10411,7 +10411,7 @@
         <v>13</v>
       </c>
       <c r="E137" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F137" s="154">
         <v>3</v>
@@ -10434,7 +10434,7 @@
     </row>
     <row r="138" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
-        <v>638</v>
+        <v>635</v>
       </c>
       <c r="B138" t="s">
         <v>236</v>
@@ -10446,7 +10446,7 @@
         <v>13</v>
       </c>
       <c r="E138" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F138" s="154">
         <v>3</v>
@@ -10481,7 +10481,7 @@
         <v>13</v>
       </c>
       <c r="E139" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F139" s="154">
         <v>5</v>
@@ -10504,7 +10504,7 @@
     </row>
     <row r="140" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
-        <v>639</v>
+        <v>636</v>
       </c>
       <c r="B140" t="s">
         <v>239</v>
@@ -10516,7 +10516,7 @@
         <v>13</v>
       </c>
       <c r="E140" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F140" s="154">
         <v>4</v>
@@ -10539,7 +10539,7 @@
     </row>
     <row r="141" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="B141" t="s">
         <v>63</v>
@@ -10551,7 +10551,7 @@
         <v>13</v>
       </c>
       <c r="E141" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F141" s="154">
         <v>4</v>
@@ -10574,7 +10574,7 @@
     </row>
     <row r="142" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
-        <v>641</v>
+        <v>638</v>
       </c>
       <c r="B142" t="s">
         <v>242</v>
@@ -10586,7 +10586,7 @@
         <v>13</v>
       </c>
       <c r="E142" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F142" s="154">
         <v>4</v>
@@ -10609,7 +10609,7 @@
     </row>
     <row r="143" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
-        <v>642</v>
+        <v>639</v>
       </c>
       <c r="B143" t="s">
         <v>197</v>
@@ -10621,7 +10621,7 @@
         <v>13</v>
       </c>
       <c r="E143" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F143" s="154">
         <v>4</v>
@@ -10644,7 +10644,7 @@
     </row>
     <row r="144" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
-        <v>643</v>
+        <v>640</v>
       </c>
       <c r="B144" t="s">
         <v>32</v>
@@ -10656,7 +10656,7 @@
         <v>13</v>
       </c>
       <c r="E144" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F144" s="154">
         <v>5</v>
@@ -10679,7 +10679,7 @@
     </row>
     <row r="145" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
-        <v>644</v>
+        <v>641</v>
       </c>
       <c r="B145" t="s">
         <v>245</v>
@@ -10691,7 +10691,7 @@
         <v>13</v>
       </c>
       <c r="E145" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F145" s="154">
         <v>2</v>
@@ -10714,7 +10714,7 @@
     </row>
     <row r="146" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
       <c r="B146" t="s">
         <v>246</v>
@@ -10726,7 +10726,7 @@
         <v>13</v>
       </c>
       <c r="E146" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F146" s="154">
         <v>5</v>
@@ -10749,7 +10749,7 @@
     </row>
     <row r="147" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
-        <v>646</v>
+        <v>643</v>
       </c>
       <c r="B147" t="s">
         <v>247</v>
@@ -10761,7 +10761,7 @@
         <v>13</v>
       </c>
       <c r="E147" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F147" s="154">
         <v>5</v>
@@ -10784,7 +10784,7 @@
     </row>
     <row r="148" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
-        <v>647</v>
+        <v>644</v>
       </c>
       <c r="B148" t="s">
         <v>184</v>
@@ -10796,7 +10796,7 @@
         <v>13</v>
       </c>
       <c r="E148" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F148" s="154">
         <v>4</v>
@@ -10819,7 +10819,7 @@
     </row>
     <row r="149" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
-        <v>648</v>
+        <v>645</v>
       </c>
       <c r="B149" t="s">
         <v>248</v>
@@ -10831,7 +10831,7 @@
         <v>13</v>
       </c>
       <c r="E149" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F149" s="154">
         <v>5</v>
@@ -10854,7 +10854,7 @@
     </row>
     <row r="150" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
       <c r="B150" t="s">
         <v>54</v>
@@ -10866,7 +10866,7 @@
         <v>13</v>
       </c>
       <c r="E150" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F150" s="154">
         <v>4</v>
@@ -10889,7 +10889,7 @@
     </row>
     <row r="151" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
-        <v>650</v>
+        <v>647</v>
       </c>
       <c r="B151" t="s">
         <v>249</v>
@@ -10901,7 +10901,7 @@
         <v>13</v>
       </c>
       <c r="E151" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F151" s="154">
         <v>4</v>
@@ -10924,7 +10924,7 @@
     </row>
     <row r="152" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
-        <v>651</v>
+        <v>648</v>
       </c>
       <c r="B152" t="s">
         <v>251</v>
@@ -10936,7 +10936,7 @@
         <v>13</v>
       </c>
       <c r="E152" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F152" s="154">
         <v>2</v>
@@ -10959,7 +10959,7 @@
     </row>
     <row r="153" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A153" t="s">
-        <v>652</v>
+        <v>649</v>
       </c>
       <c r="B153" t="s">
         <v>182</v>
@@ -10971,7 +10971,7 @@
         <v>72</v>
       </c>
       <c r="E153" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F153" s="154">
         <v>2</v>
@@ -10994,7 +10994,7 @@
     </row>
     <row r="154" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
-        <v>653</v>
+        <v>650</v>
       </c>
       <c r="B154" t="s">
         <v>56</v>
@@ -11006,7 +11006,7 @@
         <v>72</v>
       </c>
       <c r="E154" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F154" s="154">
         <v>2</v>
@@ -11029,7 +11029,7 @@
     </row>
     <row r="155" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
-        <v>654</v>
+        <v>651</v>
       </c>
       <c r="B155" t="s">
         <v>255</v>
@@ -11041,7 +11041,7 @@
         <v>72</v>
       </c>
       <c r="E155" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F155" s="154">
         <v>5</v>
@@ -11064,7 +11064,7 @@
     </row>
     <row r="156" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
-        <v>655</v>
+        <v>652</v>
       </c>
       <c r="B156" t="s">
         <v>257</v>
@@ -11076,7 +11076,7 @@
         <v>72</v>
       </c>
       <c r="E156" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F156" s="154">
         <v>4</v>
@@ -11099,7 +11099,7 @@
     </row>
     <row r="157" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
-        <v>656</v>
+        <v>653</v>
       </c>
       <c r="B157" t="s">
         <v>67</v>
@@ -11111,7 +11111,7 @@
         <v>72</v>
       </c>
       <c r="E157" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F157" s="154">
         <v>2</v>
@@ -11134,7 +11134,7 @@
     </row>
     <row r="158" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A158" t="s">
-        <v>657</v>
+        <v>654</v>
       </c>
       <c r="B158" t="s">
         <v>218</v>
@@ -11146,7 +11146,7 @@
         <v>72</v>
       </c>
       <c r="E158" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F158" s="154">
         <v>2</v>
@@ -11169,7 +11169,7 @@
     </row>
     <row r="159" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
-        <v>658</v>
+        <v>655</v>
       </c>
       <c r="B159" t="s">
         <v>259</v>
@@ -11181,7 +11181,7 @@
         <v>72</v>
       </c>
       <c r="E159" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F159" s="154">
         <v>4</v>
@@ -11204,7 +11204,7 @@
     </row>
     <row r="160" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
-        <v>659</v>
+        <v>656</v>
       </c>
       <c r="B160" t="s">
         <v>260</v>
@@ -11216,7 +11216,7 @@
         <v>72</v>
       </c>
       <c r="E160" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F160" s="154">
         <v>2</v>
@@ -11239,7 +11239,7 @@
     </row>
     <row r="161" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
-        <v>660</v>
+        <v>657</v>
       </c>
       <c r="B161" t="s">
         <v>262</v>
@@ -11251,7 +11251,7 @@
         <v>72</v>
       </c>
       <c r="E161" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F161" s="154">
         <v>4</v>
@@ -11274,7 +11274,7 @@
     </row>
     <row r="162" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A162" t="s">
-        <v>661</v>
+        <v>658</v>
       </c>
       <c r="B162" t="s">
         <v>98</v>
@@ -11286,7 +11286,7 @@
         <v>72</v>
       </c>
       <c r="E162" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F162" s="154">
         <v>5</v>
@@ -11309,7 +11309,7 @@
     </row>
     <row r="163" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A163" t="s">
-        <v>662</v>
+        <v>659</v>
       </c>
       <c r="B163" t="s">
         <v>264</v>
@@ -11321,7 +11321,7 @@
         <v>72</v>
       </c>
       <c r="E163" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F163" s="154">
         <v>3</v>
@@ -11344,7 +11344,7 @@
     </row>
     <row r="164" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A164" t="s">
-        <v>663</v>
+        <v>660</v>
       </c>
       <c r="B164" t="s">
         <v>266</v>
@@ -11356,7 +11356,7 @@
         <v>72</v>
       </c>
       <c r="E164" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F164" s="154">
         <v>5</v>
@@ -11379,7 +11379,7 @@
     </row>
     <row r="165" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A165" t="s">
-        <v>664</v>
+        <v>661</v>
       </c>
       <c r="B165" t="s">
         <v>267</v>
@@ -11391,7 +11391,7 @@
         <v>72</v>
       </c>
       <c r="E165" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F165" s="154">
         <v>5</v>
@@ -11414,7 +11414,7 @@
     </row>
     <row r="166" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A166" t="s">
-        <v>665</v>
+        <v>662</v>
       </c>
       <c r="B166" t="s">
         <v>268</v>
@@ -11426,7 +11426,7 @@
         <v>72</v>
       </c>
       <c r="E166" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F166" s="154">
         <v>3</v>
@@ -11449,7 +11449,7 @@
     </row>
     <row r="167" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A167" t="s">
-        <v>666</v>
+        <v>663</v>
       </c>
       <c r="B167" t="s">
         <v>270</v>
@@ -11461,7 +11461,7 @@
         <v>72</v>
       </c>
       <c r="E167" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F167" s="154">
         <v>4</v>
@@ -11484,7 +11484,7 @@
     </row>
     <row r="168" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A168" t="s">
-        <v>667</v>
+        <v>664</v>
       </c>
       <c r="B168" t="s">
         <v>271</v>
@@ -11496,7 +11496,7 @@
         <v>72</v>
       </c>
       <c r="E168" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F168" s="154">
         <v>4</v>
@@ -11519,7 +11519,7 @@
     </row>
     <row r="169" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A169" t="s">
-        <v>668</v>
+        <v>665</v>
       </c>
       <c r="B169" t="s">
         <v>273</v>
@@ -11531,7 +11531,7 @@
         <v>72</v>
       </c>
       <c r="E169" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F169" s="154">
         <v>5</v>
@@ -11554,7 +11554,7 @@
     </row>
     <row r="170" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A170" t="s">
-        <v>669</v>
+        <v>666</v>
       </c>
       <c r="B170" t="s">
         <v>200</v>
@@ -11566,7 +11566,7 @@
         <v>72</v>
       </c>
       <c r="E170" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F170" s="154">
         <v>2</v>
@@ -11589,7 +11589,7 @@
     </row>
     <row r="171" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A171" t="s">
-        <v>670</v>
+        <v>667</v>
       </c>
       <c r="B171" t="s">
         <v>276</v>
@@ -11601,7 +11601,7 @@
         <v>72</v>
       </c>
       <c r="E171" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F171" s="154">
         <v>2</v>
@@ -11624,7 +11624,7 @@
     </row>
     <row r="172" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A172" t="s">
-        <v>671</v>
+        <v>668</v>
       </c>
       <c r="B172" t="s">
         <v>277</v>
@@ -11636,7 +11636,7 @@
         <v>72</v>
       </c>
       <c r="E172" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F172" s="154">
         <v>2</v>
@@ -11659,7 +11659,7 @@
     </row>
     <row r="173" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A173" t="s">
-        <v>672</v>
+        <v>669</v>
       </c>
       <c r="B173" t="s">
         <v>270</v>
@@ -11671,7 +11671,7 @@
         <v>72</v>
       </c>
       <c r="E173" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F173" s="154">
         <v>3</v>
@@ -11694,7 +11694,7 @@
     </row>
     <row r="174" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A174" t="s">
-        <v>676</v>
+        <v>673</v>
       </c>
       <c r="B174" t="s">
         <v>279</v>
@@ -11706,7 +11706,7 @@
         <v>72</v>
       </c>
       <c r="E174" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F174" s="154">
         <v>5</v>
@@ -11729,7 +11729,7 @@
     </row>
     <row r="175" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A175" t="s">
-        <v>673</v>
+        <v>670</v>
       </c>
       <c r="B175" t="s">
         <v>98</v>
@@ -11741,7 +11741,7 @@
         <v>72</v>
       </c>
       <c r="E175" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F175" s="154">
         <v>3</v>
@@ -11764,7 +11764,7 @@
     </row>
     <row r="176" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A176" t="s">
-        <v>674</v>
+        <v>671</v>
       </c>
       <c r="B176" t="s">
         <v>282</v>
@@ -11776,7 +11776,7 @@
         <v>72</v>
       </c>
       <c r="E176" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F176" s="154">
         <v>5</v>
@@ -11799,7 +11799,7 @@
     </row>
     <row r="177" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A177" t="s">
-        <v>675</v>
+        <v>672</v>
       </c>
       <c r="B177" t="s">
         <v>284</v>
@@ -11811,7 +11811,7 @@
         <v>72</v>
       </c>
       <c r="E177" t="s">
-        <v>504</v>
+        <v>676</v>
       </c>
       <c r="F177" s="154">
         <v>3</v>
@@ -47088,6 +47088,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008E9E3C8083B0BC408EA3784C56B7F01C" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="aef9c2e09ffa447319707844ce559c7b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="546679d2-2e3f-4cf2-b41e-29ea27dcf39d" xmlns:ns4="250a7ea4-ef27-4a02-940c-2430205c3312" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6ba0dd40ba81b7a683c2605a999c8e51" ns3:_="" ns4:_="">
     <xsd:import namespace="546679d2-2e3f-4cf2-b41e-29ea27dcf39d"/>
@@ -47332,15 +47341,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -47350,6 +47350,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DAE25A3B-249C-477D-8D6A-46DCEEA05125}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C8FCC7B7-DA2C-4DFC-A2B0-70FB034A011D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -47364,14 +47372,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DAE25A3B-249C-477D-8D6A-46DCEEA05125}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Actualizacion de Datos Final
</commit_message>
<xml_diff>
--- a/data/CORTEPRIMERSEMESTRE2026.xlsx
+++ b/data/CORTEPRIMERSEMESTRE2026.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\IT Teacher\Documents\BOLETINES\Corte de Calificaciones\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E62648DD-20A8-4D56-9EE5-9C2CA6E4173B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C13927F0-96D3-45BA-92ED-B649DB89E800}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="11370" xr2:uid="{A1D48B81-9DDC-468E-92F8-F1A357059321}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{A1D48B81-9DDC-468E-92F8-F1A357059321}"/>
   </bookViews>
   <sheets>
     <sheet name="DB" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
-    <sheet name="Sheet4" sheetId="4" r:id="rId4"/>
+    <sheet name="Sheet2" sheetId="2" state="hidden" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" state="hidden" r:id="rId3"/>
+    <sheet name="Sheet4" sheetId="4" state="hidden" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -5694,6 +5694,9 @@
       <c r="F2" s="154">
         <v>3.75</v>
       </c>
+      <c r="G2" s="154">
+        <v>4.8</v>
+      </c>
       <c r="H2" s="154">
         <v>5</v>
       </c>
@@ -5726,6 +5729,9 @@
       <c r="F3" s="154">
         <v>4.2249999999999996</v>
       </c>
+      <c r="G3" s="154">
+        <v>4.8</v>
+      </c>
       <c r="H3" s="154">
         <v>4.8860000000000001</v>
       </c>
@@ -5758,6 +5764,9 @@
       <c r="F4" s="154">
         <v>3.875</v>
       </c>
+      <c r="G4" s="154">
+        <v>4.7</v>
+      </c>
       <c r="H4" s="154">
         <v>4.0360000000000005</v>
       </c>
@@ -5790,6 +5799,9 @@
       <c r="F5" s="154">
         <v>4.625</v>
       </c>
+      <c r="G5" s="154">
+        <v>5</v>
+      </c>
       <c r="H5" s="154">
         <v>5</v>
       </c>
@@ -5822,6 +5834,9 @@
       <c r="F6" s="154">
         <v>3.5</v>
       </c>
+      <c r="G6" s="154">
+        <v>4.8</v>
+      </c>
       <c r="H6" s="154">
         <v>5</v>
       </c>
@@ -5854,6 +5869,9 @@
       <c r="F7" s="154">
         <v>3.8499999999999996</v>
       </c>
+      <c r="G7" s="154">
+        <v>4.5999999999999996</v>
+      </c>
       <c r="H7" s="154">
         <v>5</v>
       </c>
@@ -5886,6 +5904,9 @@
       <c r="F8" s="154">
         <v>3.5</v>
       </c>
+      <c r="G8" s="154">
+        <v>4.8</v>
+      </c>
       <c r="H8" s="154">
         <v>4.97</v>
       </c>
@@ -5918,6 +5939,9 @@
       <c r="F9" s="154">
         <v>4.125</v>
       </c>
+      <c r="G9" s="154">
+        <v>4.7</v>
+      </c>
       <c r="H9" s="154">
         <v>5</v>
       </c>
@@ -5950,6 +5974,9 @@
       <c r="F10" s="154">
         <v>4.05</v>
       </c>
+      <c r="G10" s="154">
+        <v>4.7</v>
+      </c>
       <c r="H10" s="154">
         <v>5</v>
       </c>
@@ -5982,6 +6009,9 @@
       <c r="F11" s="154">
         <v>4.3250000000000002</v>
       </c>
+      <c r="G11" s="154">
+        <v>4.5999999999999996</v>
+      </c>
       <c r="H11" s="154">
         <v>5</v>
       </c>
@@ -6014,6 +6044,9 @@
       <c r="F12" s="154">
         <v>4.3</v>
       </c>
+      <c r="G12" s="154">
+        <v>4.3</v>
+      </c>
       <c r="H12" s="154">
         <v>4.79</v>
       </c>
@@ -6046,6 +6079,9 @@
       <c r="F13" s="154">
         <v>4.4750000000000005</v>
       </c>
+      <c r="G13" s="154">
+        <v>4.7</v>
+      </c>
       <c r="H13" s="154">
         <v>5</v>
       </c>
@@ -6078,6 +6114,9 @@
       <c r="F14" s="154">
         <v>4.1749999999999998</v>
       </c>
+      <c r="G14" s="154">
+        <v>4.9000000000000004</v>
+      </c>
       <c r="H14" s="154">
         <v>5</v>
       </c>
@@ -6110,6 +6149,9 @@
       <c r="F15" s="154">
         <v>3.6749999999999998</v>
       </c>
+      <c r="G15" s="154">
+        <v>4.8</v>
+      </c>
       <c r="H15" s="154">
         <v>4.8860000000000001</v>
       </c>
@@ -6142,6 +6184,9 @@
       <c r="F16" s="154">
         <v>4.1999999999999993</v>
       </c>
+      <c r="G16" s="154">
+        <v>4.5999999999999996</v>
+      </c>
       <c r="H16" s="154">
         <v>4.91</v>
       </c>
@@ -6174,6 +6219,9 @@
       <c r="F17" s="154">
         <v>4.3499999999999996</v>
       </c>
+      <c r="G17" s="154">
+        <v>4.3</v>
+      </c>
       <c r="H17" s="154">
         <v>5</v>
       </c>
@@ -6206,6 +6254,9 @@
       <c r="F18" s="154">
         <v>3.9749999999999996</v>
       </c>
+      <c r="G18" s="154">
+        <v>4.8</v>
+      </c>
       <c r="H18" s="154">
         <v>5</v>
       </c>
@@ -6238,6 +6289,9 @@
       <c r="F19" s="154">
         <v>4.0999999999999996</v>
       </c>
+      <c r="G19" s="154">
+        <v>4.7</v>
+      </c>
       <c r="H19" s="154">
         <v>5</v>
       </c>
@@ -6270,6 +6324,9 @@
       <c r="F20" s="154">
         <v>4.5</v>
       </c>
+      <c r="G20" s="154">
+        <v>4.7</v>
+      </c>
       <c r="H20" s="154">
         <v>5</v>
       </c>
@@ -6302,6 +6359,9 @@
       <c r="F21" s="154">
         <v>4.3499999999999996</v>
       </c>
+      <c r="G21" s="154">
+        <v>4.8</v>
+      </c>
       <c r="H21" s="154">
         <v>5</v>
       </c>
@@ -6334,6 +6394,9 @@
       <c r="F22" s="154">
         <v>3.4499999999999997</v>
       </c>
+      <c r="G22" s="154">
+        <v>4.7</v>
+      </c>
       <c r="H22" s="154">
         <v>5</v>
       </c>
@@ -6366,6 +6429,9 @@
       <c r="F23" s="154">
         <v>3.95</v>
       </c>
+      <c r="G23" s="154">
+        <v>4.5</v>
+      </c>
       <c r="H23" s="154">
         <v>4.8860000000000001</v>
       </c>
@@ -6398,6 +6464,9 @@
       <c r="F24" s="154">
         <v>4.375</v>
       </c>
+      <c r="G24" s="154">
+        <v>4.8</v>
+      </c>
       <c r="H24" s="154">
         <v>5</v>
       </c>
@@ -6430,6 +6499,9 @@
       <c r="F25" s="154">
         <v>4.5999999999999996</v>
       </c>
+      <c r="G25" s="154">
+        <v>4.8</v>
+      </c>
       <c r="H25" s="154">
         <v>4.9399999999999995</v>
       </c>
@@ -6462,6 +6534,9 @@
       <c r="F26" s="154">
         <v>4.5750000000000002</v>
       </c>
+      <c r="G26" s="154">
+        <v>4.9000000000000004</v>
+      </c>
       <c r="H26" s="154">
         <v>5</v>
       </c>
@@ -6494,6 +6569,9 @@
       <c r="F27" s="154">
         <v>4.4499999999999993</v>
       </c>
+      <c r="G27" s="154">
+        <v>4.5999999999999996</v>
+      </c>
       <c r="H27" s="154">
         <v>5</v>
       </c>
@@ -6526,6 +6604,9 @@
       <c r="F28" s="154">
         <v>3.875</v>
       </c>
+      <c r="G28" s="154">
+        <v>4.8</v>
+      </c>
       <c r="H28" s="154">
         <v>5</v>
       </c>
@@ -6558,6 +6639,9 @@
       <c r="F29" s="154">
         <v>3.9249999999999998</v>
       </c>
+      <c r="G29" s="154">
+        <v>4.7</v>
+      </c>
       <c r="H29" s="154">
         <v>5</v>
       </c>
@@ -6590,6 +6674,9 @@
       <c r="F30" s="154">
         <v>4.125</v>
       </c>
+      <c r="G30" s="154">
+        <v>4.7</v>
+      </c>
       <c r="H30" s="154">
         <v>4.8860000000000001</v>
       </c>
@@ -6622,6 +6709,9 @@
       <c r="F31" s="154">
         <v>3.3</v>
       </c>
+      <c r="G31" s="154">
+        <v>4.5999999999999996</v>
+      </c>
       <c r="H31" s="154">
         <v>5</v>
       </c>
@@ -6654,6 +6744,9 @@
       <c r="F32" s="154">
         <v>4.1749999999999998</v>
       </c>
+      <c r="G32" s="154">
+        <v>4.7</v>
+      </c>
       <c r="H32" s="154">
         <v>5</v>
       </c>
@@ -6686,6 +6779,9 @@
       <c r="F33" s="154">
         <v>4.05</v>
       </c>
+      <c r="G33" s="154">
+        <v>4.5</v>
+      </c>
       <c r="H33" s="154">
         <v>5</v>
       </c>
@@ -6718,6 +6814,9 @@
       <c r="F34" s="155">
         <v>4.2249999999999996</v>
       </c>
+      <c r="G34" s="154">
+        <v>4.8</v>
+      </c>
       <c r="H34" s="155">
         <v>5</v>
       </c>
@@ -6750,6 +6849,9 @@
       <c r="F35" s="155">
         <v>4.6499999999999995</v>
       </c>
+      <c r="G35" s="154">
+        <v>4.7</v>
+      </c>
       <c r="H35" s="155">
         <v>5</v>
       </c>
@@ -6782,6 +6884,9 @@
       <c r="F36" s="155">
         <v>3.9749999999999996</v>
       </c>
+      <c r="G36" s="154">
+        <v>4.8</v>
+      </c>
       <c r="H36" s="155">
         <v>5</v>
       </c>
@@ -6814,6 +6919,9 @@
       <c r="F37" s="155">
         <v>3.8</v>
       </c>
+      <c r="G37" s="154">
+        <v>4.8</v>
+      </c>
       <c r="H37" s="155">
         <v>3.2</v>
       </c>
@@ -6846,6 +6954,9 @@
       <c r="F38" s="155">
         <v>4.4249999999999998</v>
       </c>
+      <c r="G38" s="154">
+        <v>4.9000000000000004</v>
+      </c>
       <c r="H38" s="155">
         <v>5</v>
       </c>
@@ -6878,6 +6989,9 @@
       <c r="F39" s="155">
         <v>4.6749999999999998</v>
       </c>
+      <c r="G39" s="154">
+        <v>4.7</v>
+      </c>
       <c r="H39" s="155">
         <v>4.91</v>
       </c>
@@ -6910,6 +7024,9 @@
       <c r="F40" s="155">
         <v>4.3999999999999995</v>
       </c>
+      <c r="G40" s="154">
+        <v>4.8</v>
+      </c>
       <c r="H40" s="155">
         <v>5</v>
       </c>
@@ -6942,6 +7059,9 @@
       <c r="F41" s="155">
         <v>4.4249999999999998</v>
       </c>
+      <c r="G41" s="154">
+        <v>4.8</v>
+      </c>
       <c r="H41" s="155">
         <v>5</v>
       </c>
@@ -6974,6 +7094,9 @@
       <c r="F42" s="155">
         <v>4.2249999999999996</v>
       </c>
+      <c r="G42" s="154">
+        <v>4.9000000000000004</v>
+      </c>
       <c r="H42" s="155">
         <v>5</v>
       </c>
@@ -7006,6 +7129,9 @@
       <c r="F43" s="155">
         <v>4.125</v>
       </c>
+      <c r="G43" s="154">
+        <v>4.7</v>
+      </c>
       <c r="H43" s="155">
         <v>4.8499999999999996</v>
       </c>
@@ -7038,6 +7164,9 @@
       <c r="F44" s="155">
         <v>4.375</v>
       </c>
+      <c r="G44" s="154">
+        <v>4.8</v>
+      </c>
       <c r="H44" s="155">
         <v>3.26</v>
       </c>
@@ -7070,6 +7199,9 @@
       <c r="F45" s="155">
         <v>3.875</v>
       </c>
+      <c r="G45" s="154">
+        <v>4.8</v>
+      </c>
       <c r="H45" s="155">
         <v>4.91</v>
       </c>
@@ -7102,6 +7234,9 @@
       <c r="F46" s="155">
         <v>4.4250000000000007</v>
       </c>
+      <c r="G46" s="154">
+        <v>4.5999999999999996</v>
+      </c>
       <c r="H46" s="155">
         <v>5</v>
       </c>
@@ -7134,6 +7269,9 @@
       <c r="F47" s="155">
         <v>4.5749999999999993</v>
       </c>
+      <c r="G47" s="154">
+        <v>4.9000000000000004</v>
+      </c>
       <c r="H47" s="155">
         <v>5</v>
       </c>
@@ -7166,6 +7304,9 @@
       <c r="F48" s="155">
         <v>4.3999999999999995</v>
       </c>
+      <c r="G48" s="154">
+        <v>4.9000000000000004</v>
+      </c>
       <c r="H48" s="155">
         <v>5</v>
       </c>
@@ -7198,6 +7339,9 @@
       <c r="F49" s="155">
         <v>4.5750000000000002</v>
       </c>
+      <c r="G49" s="154">
+        <v>4.9000000000000004</v>
+      </c>
       <c r="H49" s="155">
         <v>5</v>
       </c>
@@ -7230,6 +7374,9 @@
       <c r="F50" s="155">
         <v>4.5750000000000002</v>
       </c>
+      <c r="G50" s="154">
+        <v>4.7</v>
+      </c>
       <c r="H50" s="155">
         <v>3.71</v>
       </c>
@@ -7259,6 +7406,9 @@
       <c r="F51" s="155">
         <v>4.4249999999999989</v>
       </c>
+      <c r="G51" s="154">
+        <v>4.8</v>
+      </c>
       <c r="H51" s="155">
         <v>5</v>
       </c>
@@ -7291,6 +7441,9 @@
       <c r="F52" s="155">
         <v>3.7749999999999995</v>
       </c>
+      <c r="G52" s="154">
+        <v>5</v>
+      </c>
       <c r="H52" s="155">
         <v>5</v>
       </c>
@@ -7323,6 +7476,9 @@
       <c r="F53" s="154">
         <v>4.6749999999999998</v>
       </c>
+      <c r="G53" s="154">
+        <v>4.8</v>
+      </c>
       <c r="H53" s="154">
         <v>5</v>
       </c>
@@ -7355,6 +7511,9 @@
       <c r="F54" s="154">
         <v>4.1749999999999998</v>
       </c>
+      <c r="G54" s="154">
+        <v>4.8</v>
+      </c>
       <c r="H54" s="154">
         <v>5</v>
       </c>
@@ -7387,6 +7546,9 @@
       <c r="F55" s="154">
         <v>4</v>
       </c>
+      <c r="G55" s="154">
+        <v>4.7</v>
+      </c>
       <c r="H55" s="154">
         <v>4.7</v>
       </c>
@@ -7419,6 +7581,9 @@
       <c r="F56" s="154">
         <v>3.7749999999999999</v>
       </c>
+      <c r="G56" s="154">
+        <v>4.5999999999999996</v>
+      </c>
       <c r="H56" s="154">
         <v>4.7</v>
       </c>
@@ -7451,6 +7616,9 @@
       <c r="F57" s="154">
         <v>3.4499999999999997</v>
       </c>
+      <c r="G57" s="154">
+        <v>4.7</v>
+      </c>
       <c r="H57" s="154">
         <v>4.7</v>
       </c>
@@ -7483,6 +7651,9 @@
       <c r="F58" s="154">
         <v>4.0749999999999993</v>
       </c>
+      <c r="G58" s="154">
+        <v>4.9000000000000004</v>
+      </c>
       <c r="H58" s="154">
         <v>4.7</v>
       </c>
@@ -7515,6 +7686,9 @@
       <c r="F59" s="154">
         <v>4.0249999999999995</v>
       </c>
+      <c r="G59" s="154">
+        <v>4.9000000000000004</v>
+      </c>
       <c r="H59" s="154">
         <v>4.7</v>
       </c>
@@ -7547,6 +7721,9 @@
       <c r="F60" s="154">
         <v>4.125</v>
       </c>
+      <c r="G60" s="154">
+        <v>4.8</v>
+      </c>
       <c r="H60" s="154">
         <v>4.7</v>
       </c>
@@ -7579,6 +7756,9 @@
       <c r="F61" s="154">
         <v>4.3250000000000002</v>
       </c>
+      <c r="G61" s="154">
+        <v>4.9000000000000004</v>
+      </c>
       <c r="H61" s="154">
         <v>4.6399999999999997</v>
       </c>
@@ -7611,6 +7791,9 @@
       <c r="F62" s="154">
         <v>4.6749999999999998</v>
       </c>
+      <c r="G62" s="154">
+        <v>4.7</v>
+      </c>
       <c r="H62" s="154">
         <v>4.7</v>
       </c>
@@ -7643,6 +7826,9 @@
       <c r="F63" s="154">
         <v>4.3499999999999996</v>
       </c>
+      <c r="G63" s="154">
+        <v>4.7</v>
+      </c>
       <c r="H63" s="154">
         <v>4.7</v>
       </c>
@@ -7921,7 +8107,7 @@
         <v>4.58</v>
       </c>
       <c r="G71" s="154">
-        <v>4.3</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="H71" s="154">
         <v>4.67</v>
@@ -8201,7 +8387,7 @@
         <v>4.62</v>
       </c>
       <c r="G79" s="154">
-        <v>4.5</v>
+        <v>4.7</v>
       </c>
       <c r="H79" s="154">
         <v>4.6999999999999993</v>
@@ -8341,7 +8527,7 @@
         <v>4.24</v>
       </c>
       <c r="G83" s="154">
-        <v>4.5</v>
+        <v>4.7</v>
       </c>
       <c r="H83" s="154">
         <v>4.8199999999999994</v>
@@ -8516,7 +8702,7 @@
         <v>4.68</v>
       </c>
       <c r="G88" s="154">
-        <v>4.3</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="H88" s="154">
         <v>4.76</v>

</xml_diff>